<commit_message>
Update New Microsoft Excel Worksheet.xlsx
</commit_message>
<xml_diff>
--- a/Extra Data/New Microsoft Excel Worksheet.xlsx
+++ b/Extra Data/New Microsoft Excel Worksheet.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\natha\OneDrive\Documents\TheEldenLords\Extra Data\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1990FF7-8FA0-4753-BBF6-91972812DE85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="20715" windowHeight="13515" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -18,8 +24,262 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="83">
+  <si>
+    <t>Bosses</t>
+  </si>
+  <si>
+    <t>Location</t>
+  </si>
+  <si>
+    <t>Lore</t>
+  </si>
+  <si>
+    <t>Stats</t>
+  </si>
+  <si>
+    <t>Prerequisites</t>
+  </si>
+  <si>
+    <t>Help</t>
+  </si>
+  <si>
+    <t>Rewards</t>
+  </si>
+  <si>
+    <t>Margit The Fell Omen</t>
+  </si>
+  <si>
+    <t>Godrick the Grafted</t>
+  </si>
+  <si>
+    <t>Rennala Queen of the Full Moon</t>
+  </si>
+  <si>
+    <t>Starscourge Radahn</t>
+  </si>
+  <si>
+    <t>Mohg Lord of Blood</t>
+  </si>
+  <si>
+    <t>Rykard Lord of Blasphemy</t>
+  </si>
+  <si>
+    <t>Draconic Tree Sentinel</t>
+  </si>
+  <si>
+    <t>Godfrey First Elden Lord (Golden Shade)</t>
+  </si>
+  <si>
+    <t>Morgott The Omen King</t>
+  </si>
+  <si>
+    <t>Fire Giant</t>
+  </si>
+  <si>
+    <t>Godskin Duo</t>
+  </si>
+  <si>
+    <t>Sir Gideon-Ofnir the All Knowing</t>
+  </si>
+  <si>
+    <t>Godfrey First Elden Lord (Hoarah Loux)</t>
+  </si>
+  <si>
+    <t>Radagon of the Golden Order</t>
+  </si>
+  <si>
+    <t>Elden Beast</t>
+  </si>
+  <si>
+    <t>Stormveil Castle</t>
+  </si>
+  <si>
+    <t>None</t>
+  </si>
+  <si>
+    <t>12,000 runes, Talisman Pouch</t>
+  </si>
+  <si>
+    <t>HP: 4174, Def: 103, Stance: 80</t>
+  </si>
+  <si>
+    <t>20,000 runes, Godrick's Great Rune, Remembrance of the Grafted</t>
+  </si>
+  <si>
+    <t>HP: 6080, Def: 105, Stance: 105</t>
+  </si>
+  <si>
+    <t>Defeat Margit The Fell Omen</t>
+  </si>
+  <si>
+    <t>Raya Lucaria Academy</t>
+  </si>
+  <si>
+    <t>40,000 Runes, Remembrance of the Full Moon, Great Rune of the Unborn</t>
+  </si>
+  <si>
+    <t>Glintstone Key, Defeat Red Wolf</t>
+  </si>
+  <si>
+    <t>Redmane Castle</t>
+  </si>
+  <si>
+    <t>HP: 9572, Def: 113, Stance: 200</t>
+  </si>
+  <si>
+    <t>Strong vs Magic - Weak to Standard, Slash, Pierce</t>
+  </si>
+  <si>
+    <t>Strong vs Holy - Weak to All Physical Damage</t>
+  </si>
+  <si>
+    <t>Strong vs Holy - Weak to Slash</t>
+  </si>
+  <si>
+    <t>Strong vs Holy, Sleep - Weak to Pierce, Scarlet Rot</t>
+  </si>
+  <si>
+    <t>70,000 Runes, Remembrance of the Starscourge, Radahn's Great Rune</t>
+  </si>
+  <si>
+    <t>Trigger Radahn Festival</t>
+  </si>
+  <si>
+    <t>1st Phase: HP: 3493, Def: 109, Stance: 0 - 2nd Phase: HP: 4097, Def: 109, Stance: 80</t>
+  </si>
+  <si>
+    <t>Mohgwyn Palace</t>
+  </si>
+  <si>
+    <t>HP: 18,389, Def: 122, Stance: 110</t>
+  </si>
+  <si>
+    <t>Strong vs Fire - Weak to All Physcial, Hemorrhage</t>
+  </si>
+  <si>
+    <t>420,000 Runes, Mohg's Great Rune, Remembrance of the Blood Lord</t>
+  </si>
+  <si>
+    <t>Pureblood Knight's Medal</t>
+  </si>
+  <si>
+    <t>Volcano Manor</t>
+  </si>
+  <si>
+    <t>Serpent: HP: 30493 - Rykard: 59174, Def: 115, Stance: 120</t>
+  </si>
+  <si>
+    <t>Strong vs Fire - Weak to All Physcial</t>
+  </si>
+  <si>
+    <t>130,000 Runes, Rykard's Great Rune, Remembrance of the Blastphemous</t>
+  </si>
+  <si>
+    <t>Capital Outskirts</t>
+  </si>
+  <si>
+    <t>Strong vs Slash, Fire, Lightning, Hemorrhage, Frostbite - Weak to Standard, Strike, Pierce</t>
+  </si>
+  <si>
+    <t>50,000 Runes, Dragon Greatclaw, Dragonclaw Shield</t>
+  </si>
+  <si>
+    <t>HP: 13362, Def: 118, Stance: 80</t>
+  </si>
+  <si>
+    <t>Leyndell, Royal Capital</t>
+  </si>
+  <si>
+    <t>HP: 7099, Def: 114, Stance: 120</t>
+  </si>
+  <si>
+    <t>Strong vs Holy - Neutral to Pierce, Lightning</t>
+  </si>
+  <si>
+    <t>80,000 runes, Tailsman Pouch</t>
+  </si>
+  <si>
+    <t>HP: 10399, Def: 114, Stance: 80</t>
+  </si>
+  <si>
+    <t>Strong vs Holy, Sleep - Weak to Slash</t>
+  </si>
+  <si>
+    <t>120,000 runes, Remembrance of the Omen King, Morgott's Great Rune, Talisman Pouch</t>
+  </si>
+  <si>
+    <t>2 Great Runes, Defeat Draconic Tree Sentinel &amp; Godfrey Golden Shade</t>
+  </si>
+  <si>
+    <t>Flame Peak</t>
+  </si>
+  <si>
+    <t>HP: 42363, Def: 118, Stance: 120</t>
+  </si>
+  <si>
+    <t>Defeat Morgott the Omen King</t>
+  </si>
+  <si>
+    <t>Strong vs Fire, Frostbite - Weak to Slash</t>
+  </si>
+  <si>
+    <t>180,00 Runes, Remembrance of the Fire Giant</t>
+  </si>
+  <si>
+    <t>Crumbling Farum Azula</t>
+  </si>
+  <si>
+    <t>Strong vs Strike, Fire, Holy - Weak to Slash, Sleep, Hemorrhage</t>
+  </si>
+  <si>
+    <t>170,000 Runes, Ash of War: Black Flame Tornado, Smithing Stone Bell Bearing [4]</t>
+  </si>
+  <si>
+    <t>Apostle: HP: 6668, Def: 118, Stance: 80 - Noble: HP: 8000, Def: 118, Stance: 80</t>
+  </si>
+  <si>
+    <t>Beast Clergyman/Maliketh The Black Blade</t>
+  </si>
+  <si>
+    <t>HP: 10620, Def: 120, Stance: 80</t>
+  </si>
+  <si>
+    <t>Strong vs Holy, Sleep - Weak to All Physical Damage</t>
+  </si>
+  <si>
+    <t>220,000 Runes, Remembrance of the Black Blade</t>
+  </si>
+  <si>
+    <t>Leyndell, Ashen Capital</t>
+  </si>
+  <si>
+    <t>Strong vs Magic - Weak to Strike, Pierce, Lightning, Sleep, Madness</t>
+  </si>
+  <si>
+    <t>150,000 Runes, All-Knowing Armor, Scepter of the All-Knowing</t>
+  </si>
+  <si>
+    <t>HP: 9312, Def: 0, Stance: 47</t>
+  </si>
+  <si>
+    <t>HP: 21903, Def: 120, Stance: 120</t>
+  </si>
+  <si>
+    <t>Defeat Gideon the All-Knowing</t>
+  </si>
+  <si>
+    <t>Strong vs Holy, Sleep - Weak to Pierce, Lightning, Slash</t>
+  </si>
+  <si>
+    <t>300,000 Runes, Remembrance of Hoarah Loux</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -330,10 +590,333 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:G17"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <cols>
+    <col min="1" max="1" width="34.796875" customWidth="1"/>
+    <col min="2" max="2" width="22.1328125" customWidth="1"/>
+    <col min="3" max="3" width="26.53125" customWidth="1"/>
+    <col min="4" max="4" width="67.3984375" customWidth="1"/>
+    <col min="5" max="5" width="56.9296875" customWidth="1"/>
+    <col min="6" max="6" width="70.53125" customWidth="1"/>
+    <col min="7" max="7" width="70.06640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D2" t="s">
+        <v>25</v>
+      </c>
+      <c r="E2" t="s">
+        <v>23</v>
+      </c>
+      <c r="F2" t="s">
+        <v>36</v>
+      </c>
+      <c r="G2" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3" t="s">
+        <v>22</v>
+      </c>
+      <c r="D3" t="s">
+        <v>27</v>
+      </c>
+      <c r="E3" t="s">
+        <v>28</v>
+      </c>
+      <c r="F3" t="s">
+        <v>35</v>
+      </c>
+      <c r="G3" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" t="s">
+        <v>29</v>
+      </c>
+      <c r="D4" t="s">
+        <v>40</v>
+      </c>
+      <c r="E4" t="s">
+        <v>31</v>
+      </c>
+      <c r="F4" t="s">
+        <v>34</v>
+      </c>
+      <c r="G4" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A5" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5" t="s">
+        <v>32</v>
+      </c>
+      <c r="D5" t="s">
+        <v>33</v>
+      </c>
+      <c r="E5" t="s">
+        <v>39</v>
+      </c>
+      <c r="F5" t="s">
+        <v>37</v>
+      </c>
+      <c r="G5" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A6" t="s">
+        <v>11</v>
+      </c>
+      <c r="B6" t="s">
+        <v>41</v>
+      </c>
+      <c r="D6" t="s">
+        <v>42</v>
+      </c>
+      <c r="E6" t="s">
+        <v>45</v>
+      </c>
+      <c r="F6" t="s">
+        <v>43</v>
+      </c>
+      <c r="G6" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A7" t="s">
+        <v>12</v>
+      </c>
+      <c r="B7" t="s">
+        <v>46</v>
+      </c>
+      <c r="D7" t="s">
+        <v>47</v>
+      </c>
+      <c r="E7" t="s">
+        <v>23</v>
+      </c>
+      <c r="F7" t="s">
+        <v>48</v>
+      </c>
+      <c r="G7" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A8" t="s">
+        <v>13</v>
+      </c>
+      <c r="B8" t="s">
+        <v>50</v>
+      </c>
+      <c r="D8" t="s">
+        <v>53</v>
+      </c>
+      <c r="E8" t="s">
+        <v>23</v>
+      </c>
+      <c r="F8" t="s">
+        <v>51</v>
+      </c>
+      <c r="G8" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A9" t="s">
+        <v>14</v>
+      </c>
+      <c r="B9" t="s">
+        <v>54</v>
+      </c>
+      <c r="D9" t="s">
+        <v>55</v>
+      </c>
+      <c r="E9" t="s">
+        <v>23</v>
+      </c>
+      <c r="F9" t="s">
+        <v>56</v>
+      </c>
+      <c r="G9" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A10" t="s">
+        <v>15</v>
+      </c>
+      <c r="B10" t="s">
+        <v>54</v>
+      </c>
+      <c r="D10" t="s">
+        <v>58</v>
+      </c>
+      <c r="E10" t="s">
+        <v>61</v>
+      </c>
+      <c r="F10" t="s">
+        <v>59</v>
+      </c>
+      <c r="G10" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A11" t="s">
+        <v>16</v>
+      </c>
+      <c r="B11" t="s">
+        <v>62</v>
+      </c>
+      <c r="D11" t="s">
+        <v>63</v>
+      </c>
+      <c r="E11" t="s">
+        <v>64</v>
+      </c>
+      <c r="F11" t="s">
+        <v>65</v>
+      </c>
+      <c r="G11" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A12" t="s">
+        <v>17</v>
+      </c>
+      <c r="B12" t="s">
+        <v>67</v>
+      </c>
+      <c r="D12" t="s">
+        <v>70</v>
+      </c>
+      <c r="E12" t="s">
+        <v>23</v>
+      </c>
+      <c r="F12" t="s">
+        <v>68</v>
+      </c>
+      <c r="G12" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A13" t="s">
+        <v>71</v>
+      </c>
+      <c r="B13" t="s">
+        <v>67</v>
+      </c>
+      <c r="D13" t="s">
+        <v>72</v>
+      </c>
+      <c r="E13" t="s">
+        <v>23</v>
+      </c>
+      <c r="F13" t="s">
+        <v>73</v>
+      </c>
+      <c r="G13" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A14" t="s">
+        <v>18</v>
+      </c>
+      <c r="B14" t="s">
+        <v>75</v>
+      </c>
+      <c r="D14" t="s">
+        <v>78</v>
+      </c>
+      <c r="E14" t="s">
+        <v>23</v>
+      </c>
+      <c r="F14" t="s">
+        <v>76</v>
+      </c>
+      <c r="G14" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A15" t="s">
+        <v>19</v>
+      </c>
+      <c r="B15" t="s">
+        <v>75</v>
+      </c>
+      <c r="D15" t="s">
+        <v>79</v>
+      </c>
+      <c r="E15" t="s">
+        <v>80</v>
+      </c>
+      <c r="F15" t="s">
+        <v>81</v>
+      </c>
+      <c r="G15" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A16" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A17" t="s">
+        <v>21</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>